<commit_message>
docs(quick-kayinleong-102): record the post-fix live re-check of P02 and P09
Re-asked on the deployed site (build d23700c, claude-sonnet-4-6): both projects are
found and answered in full, and every field they state matches the client Excel
(P02 8/8, P09 11/11). The Client Sheet Field Check rows for P02 and P09 now hold the
re-check (Pass); the sheet reads 78 Pass, 1 Partial, 4 Fail.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/UAT-Output-Test-Cases-RESULTS.xlsx
+++ b/docs/UAT-Output-Test-Cases-RESULTS.xlsx
@@ -762,7 +762,7 @@
     <row r="1">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>Each cell = one field of one project in the client's Excel (_D2 Project Info.xlsx), as answered by the LIVE site's Finder (cy-csaiagent hosted app, build 5d27801, model claude-sonnet-4-6) on 28 Oct 2026. Latest; replaces the earlier results.</t>
+          <t>Each cell = one field of one project in the client's Excel (_D2 Project Info.xlsx), as answered by the LIVE site's Finder (cy-csaiagent hosted app, build 5d27801, model claude-sonnet-4-6) on 28 Oct 2026; P02 and P09 re-asked on build d23700c after the quick-kayinleong-102 fix. Latest; replaces the earlier results.</t>
         </is>
       </c>
     </row>
@@ -984,34 +984,34 @@
           <t>PDH: Imperial Residences RA</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="E8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="F8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="G8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="H8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
+      <c r="C8" s="42" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I8" s="44" t="inlineStr">
@@ -1019,14 +1019,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="K8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
+      <c r="J8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L8" s="44" t="inlineStr">
@@ -1044,9 +1044,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O8" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
+      <c r="O8" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P8" s="44" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="S8" s="39" t="inlineStr">
         <is>
-          <t>The bot told the agent the project does not exist: it skipped searchProjects and called projectDetail with an invented ID ('pdh-imperial-residences-ra'), which matched nothing. The project is live (run 3 answered it in full). Cause (found in quick-kayinleong-102): with no search result to copy an ID from, the model built one from the project name. Fixed in quick-kayinleong-102, not yet on the live site: projectDetail now looks a project up by its exact name and, when that misses, the bot searches by name before saying anything is missing. Re-run through the real Finder agent on claude-sonnet-4-6 (28 Oct): found by name and answered in full; 7 of the 8 fields stated match the Excel. H1A bedrooms differ: the answer says '3 + Studio (Dual Key)', the Excel says 4+1.</t>
+          <t>Re-asked on the live site after the fix (build d23700c, 28 Oct): found the project and answered in full; every field it stated matches the Excel. The first run 4 answer (build 5d27801) said the project did not exist: with no search result to copy an ID from, the model built one from the name. Fixed in quick-kayinleong-102: projectDetail finds a project by its exact name, and a miss sends the bot to search by name first.</t>
         </is>
       </c>
     </row>
@@ -1633,69 +1633,69 @@
           <t>PDH: Royal Suites(RC)</t>
         </is>
       </c>
-      <c r="C15" s="45" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="E15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="F15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="G15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="H15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="I15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="J15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="K15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="L15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="M15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="N15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
-        </is>
-      </c>
-      <c r="O15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F15" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P15" s="44" t="inlineStr">
@@ -1703,9 +1703,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q15" s="46" t="inlineStr">
-        <is>
-          <t>NOT STATED</t>
+      <c r="Q15" s="43" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R15" s="44" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="S15" s="39" t="inlineStr">
         <is>
-          <t>Same as P02: the bot said 'PDH: Royal Suites (RC) does not exist in the D2 inventory system under that ID' after calling projectDetail with an invented ID. The project is live (run 3 answered it in full). Cause (found in quick-kayinleong-102): with no search result to copy an ID from, the model built one from the project name. Fixed in quick-kayinleong-102, not yet on the live site: projectDetail now looks a project up by its exact name and, when that misses, the bot searches by name before saying anything is missing. Re-run through the real Finder agent on claude-sonnet-4-6 (28 Oct): the exact name missed (it is stored as 'Pavilion Damansara Heights: Royal Suites(RC)'), the bot searched, found it and answered; all 11 fields stated match the Excel.</t>
+          <t>Re-asked on the live site after the fix (build d23700c, 28 Oct): found the project (stored as 'Pavilion Damansara Heights: Royal Suites(RC)') and answered in full; every field it stated matches the Excel. The first run 4 answer (build 5d27801) said the project did not exist: with no search result to copy an ID from, the model built one from the name. Fixed in quick-kayinleong-102: projectDetail finds a project by its exact name, and a miss sends the bot to search by name first.</t>
         </is>
       </c>
     </row>

</xml_diff>